<commit_message>
dados(entrega): regenera com V00237 e os indicadores do banheiro graduado
Banco de 105 para 108 colunas (as 3 novas: V00237, pct_so_sanitario,
pct_banheiro_comum); as 105 colunas antigas conferidas identicas por valor ao
HEAD anterior (script de comparacao, nao versionado). Base bruta do NB01 sobe
de 73 para 74 colunas. Quadro_Indicadores e Dicionario_Variaveis_Projeto
regerados a partir do codigo (scripts/gerar_quadro_indicadores.py e
scripts/gerar_tabela_variaveis.py); banheiro_particao.csv e a saida do script
de auditoria do commit anterior.
</commit_message>
<xml_diff>
--- a/banco_de_dados/entrega_orientadora/Quadro_Indicadores.xlsx
+++ b/banco_de_dados/entrega_orientadora/Quadro_Indicadores.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="120">
   <si>
     <t>indicador</t>
   </si>
@@ -100,6 +100,12 @@
     <t>pct_sem_banheiro_nem_sanitario</t>
   </si>
   <si>
+    <t>pct_so_sanitario</t>
+  </si>
+  <si>
+    <t>pct_banheiro_comum</t>
+  </si>
+  <si>
     <t>pct_resp_feminino</t>
   </si>
   <si>
@@ -196,6 +202,12 @@
     <t>Proporção de domicílios sem banheiro nem sanitário</t>
   </si>
   <si>
+    <t>Proporção de domicílios com apenas sanitário ou buraco para dejeções</t>
+  </si>
+  <si>
+    <t>Proporção de domicílios com apenas banheiro de uso comum</t>
+  </si>
+  <si>
     <t>Proporção de domicílios com pessoa responsável do sexo feminino</t>
   </si>
   <si>
@@ -272,6 +284,12 @@
   </si>
   <si>
     <t>V00238 — Domicílios Particulares Permanentes Ocupados, Não tinham banheiro nem sanitário</t>
+  </si>
+  <si>
+    <t>V00237 — Domicílios Particulares Permanentes Ocupados, Apenas sanitário ou buraco para dejeções, inclusive os localizados no terreno</t>
+  </si>
+  <si>
+    <t>V00236 — Domicílios Particulares Permanentes Ocupados, Apenas banheiro de uso comum a mais de um domicílio</t>
   </si>
   <si>
     <t>V01063 — Pessoa responsável pelo domicílio, Sexo feminino</t>
@@ -687,7 +705,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="26.7109375" customWidth="1"/>
@@ -731,28 +749,28 @@
         <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E2" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="F2" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="G2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H2" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="I2" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -760,28 +778,28 @@
         <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D3" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E3" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="F3" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="G3" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H3" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="I3" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -789,28 +807,28 @@
         <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E4" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F4" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="G4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H4" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="I4" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -818,28 +836,28 @@
         <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E5" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F5" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="G5" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H5" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="I5" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -847,28 +865,28 @@
         <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E6" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="F6" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="G6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H6" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="I6" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -876,28 +894,28 @@
         <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C7" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D7" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E7" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="F7" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H7" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="I7" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -905,28 +923,28 @@
         <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E8" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="F8" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="G8" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="I8" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -934,28 +952,28 @@
         <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D9" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E9" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="F9" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="G9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H9" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="I9" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -963,28 +981,28 @@
         <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C10" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E10" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="F10" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="G10" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H10" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="I10" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -992,28 +1010,28 @@
         <v>18</v>
       </c>
       <c r="B11" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C11" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D11" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E11" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F11" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="G11" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H11" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="I11" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -1021,28 +1039,28 @@
         <v>19</v>
       </c>
       <c r="B12" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C12" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D12" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E12" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="F12" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="G12" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H12" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="I12" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -1050,28 +1068,28 @@
         <v>20</v>
       </c>
       <c r="B13" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C13" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D13" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E13" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="F13" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="G13" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H13" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="I13" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -1079,28 +1097,28 @@
         <v>21</v>
       </c>
       <c r="B14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D14" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E14" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="F14" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="G14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H14" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="I14" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -1108,28 +1126,28 @@
         <v>22</v>
       </c>
       <c r="B15" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C15" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D15" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E15" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="F15" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="G15" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H15" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="I15" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -1137,28 +1155,28 @@
         <v>23</v>
       </c>
       <c r="B16" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C16" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D16" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E16" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="F16" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="G16" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H16" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="I16" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -1166,28 +1184,28 @@
         <v>24</v>
       </c>
       <c r="B17" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C17" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D17" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E17" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="F17" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="G17" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H17" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="I17" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -1195,28 +1213,28 @@
         <v>25</v>
       </c>
       <c r="B18" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C18" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D18" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E18" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="F18" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="G18" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H18" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="I18" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -1224,28 +1242,28 @@
         <v>26</v>
       </c>
       <c r="B19" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C19" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D19" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E19" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F19" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="G19" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H19" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="I19" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -1253,28 +1271,28 @@
         <v>27</v>
       </c>
       <c r="B20" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C20" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D20" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E20" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="F20" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="G20" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H20" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="I20" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="21" spans="1:9">
@@ -1282,28 +1300,28 @@
         <v>28</v>
       </c>
       <c r="B21" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C21" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D21" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E21" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="F21" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G21" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H21" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="I21" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -1311,28 +1329,28 @@
         <v>29</v>
       </c>
       <c r="B22" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C22" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D22" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E22" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="F22" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G22" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H22" t="s">
         <v>104</v>
       </c>
       <c r="I22" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -1343,25 +1361,25 @@
         <v>38</v>
       </c>
       <c r="C23" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D23" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E23" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="F23" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="G23" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H23" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="I23" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -1369,28 +1387,28 @@
         <v>31</v>
       </c>
       <c r="B24" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C24" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D24" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E24" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="F24" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="G24" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H24" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="I24" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -1398,25 +1416,25 @@
         <v>32</v>
       </c>
       <c r="B25" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C25" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D25" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E25" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="F25" t="s">
-        <v>88</v>
+        <v>101</v>
       </c>
       <c r="G25" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H25" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="I25" t="s">
         <v>112</v>
@@ -1427,25 +1445,25 @@
         <v>33</v>
       </c>
       <c r="B26" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C26" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D26" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E26" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="F26" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G26" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H26" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="I26" t="s">
         <v>112</v>
@@ -1456,28 +1474,86 @@
         <v>34</v>
       </c>
       <c r="B27" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C27" t="s">
+        <v>42</v>
+      </c>
+      <c r="D27" t="s">
+        <v>68</v>
+      </c>
+      <c r="E27" t="s">
+        <v>95</v>
+      </c>
+      <c r="F27" t="s">
+        <v>94</v>
+      </c>
+      <c r="G27" t="s">
+        <v>42</v>
+      </c>
+      <c r="H27" t="s">
+        <v>111</v>
+      </c>
+      <c r="I27" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9">
+      <c r="A28" t="s">
+        <v>35</v>
+      </c>
+      <c r="B28" t="s">
         <v>40</v>
       </c>
-      <c r="D27" t="s">
-        <v>66</v>
-      </c>
-      <c r="E27" t="s">
-        <v>90</v>
-      </c>
-      <c r="F27" t="s">
-        <v>89</v>
-      </c>
-      <c r="G27" t="s">
+      <c r="C28" t="s">
+        <v>42</v>
+      </c>
+      <c r="D28" t="s">
+        <v>69</v>
+      </c>
+      <c r="E28" t="s">
+        <v>95</v>
+      </c>
+      <c r="F28" t="s">
+        <v>103</v>
+      </c>
+      <c r="G28" t="s">
+        <v>42</v>
+      </c>
+      <c r="H28" t="s">
+        <v>111</v>
+      </c>
+      <c r="I28" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9">
+      <c r="A29" t="s">
+        <v>36</v>
+      </c>
+      <c r="B29" t="s">
         <v>40</v>
       </c>
-      <c r="H27" t="s">
-        <v>105</v>
-      </c>
-      <c r="I27" t="s">
-        <v>113</v>
+      <c r="C29" t="s">
+        <v>42</v>
+      </c>
+      <c r="D29" t="s">
+        <v>70</v>
+      </c>
+      <c r="E29" t="s">
+        <v>96</v>
+      </c>
+      <c r="F29" t="s">
+        <v>95</v>
+      </c>
+      <c r="G29" t="s">
+        <v>42</v>
+      </c>
+      <c r="H29" t="s">
+        <v>111</v>
+      </c>
+      <c r="I29" t="s">
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>